<commit_message>
Add logs and updated training code
</commit_message>
<xml_diff>
--- a/test_results.xlsx
+++ b/test_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wwr01\Point-Cloud-Classification-Using-PointNet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D02A4F6-2F61-4F62-BE2D-D74E5F96DF02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9041242-62CB-4030-B820-DA44D6313DFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -951,12 +951,12 @@
         <v>0.88260300000000003</v>
       </c>
       <c r="D24" s="2">
-        <f>B24-$B$2</f>
-        <v>3.4480999999999984E-2</v>
+        <f>B24-$B$24</f>
+        <v>0</v>
       </c>
       <c r="E24" s="2">
-        <f>C24-$C$2</f>
-        <v>5.5250000000000021E-2</v>
+        <f>C24-$C$24</f>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
@@ -970,12 +970,12 @@
         <v>0.878467</v>
       </c>
       <c r="D25">
-        <f>B25-$B$2</f>
-        <v>1.538700000000004E-2</v>
+        <f>B25-$B$24</f>
+        <v>-1.9093999999999944E-2</v>
       </c>
       <c r="E25">
-        <f>D25-$D$2</f>
-        <v>1.538700000000004E-2</v>
+        <f>C25-$C$24</f>
+        <v>-4.1360000000000285E-3</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
@@ -989,12 +989,12 @@
         <v>0.88206300000000004</v>
       </c>
       <c r="D26">
-        <f>B26-$B$2</f>
-        <v>2.6795000000000013E-2</v>
+        <f>B26-$B$24</f>
+        <v>-7.6859999999999706E-3</v>
       </c>
       <c r="E26">
-        <f t="shared" ref="E26" si="15">C26-$C$2</f>
-        <v>5.4710000000000036E-2</v>
+        <f>C26-$C$24</f>
+        <v>-5.3999999999998494E-4</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
@@ -1008,12 +1008,12 @@
         <v>0.88076100000000002</v>
       </c>
       <c r="D27">
-        <f t="shared" ref="D27:D31" si="16">B27-$B$2</f>
-        <v>3.3753000000000033E-2</v>
+        <f>B27-$B$24</f>
+        <v>-7.2799999999995091E-4</v>
       </c>
       <c r="E27">
-        <f t="shared" ref="E27" si="17">D27-$D$2</f>
-        <v>3.3753000000000033E-2</v>
+        <f>C27-$C$24</f>
+        <v>-1.8420000000000103E-3</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
@@ -1027,12 +1027,12 @@
         <v>0.88681200000000004</v>
       </c>
       <c r="D28">
-        <f t="shared" si="16"/>
-        <v>3.8931000000000049E-2</v>
+        <f>B28-$B$24</f>
+        <v>4.450000000000065E-3</v>
       </c>
       <c r="E28">
-        <f t="shared" ref="E28" si="18">C28-$C$2</f>
-        <v>5.945900000000004E-2</v>
+        <f>C28-$C$24</f>
+        <v>4.2090000000000183E-3</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
@@ -1046,12 +1046,12 @@
         <v>0.88156000000000001</v>
       </c>
       <c r="D29">
-        <f t="shared" si="16"/>
-        <v>3.7797999999999998E-2</v>
+        <f>B29-$B$24</f>
+        <v>3.3170000000000144E-3</v>
       </c>
       <c r="E29">
-        <f t="shared" ref="E29" si="19">D29-$D$2</f>
-        <v>3.7797999999999998E-2</v>
+        <f>C29-$C$24</f>
+        <v>-1.0430000000000161E-3</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
@@ -1065,12 +1065,12 @@
         <v>0.88656699999999999</v>
       </c>
       <c r="D30">
-        <f t="shared" si="16"/>
-        <v>3.2135000000000025E-2</v>
+        <f>B30-$B$24</f>
+        <v>-2.3459999999999592E-3</v>
       </c>
       <c r="E30">
-        <f t="shared" ref="E30" si="20">C30-$C$2</f>
-        <v>5.9213999999999989E-2</v>
+        <f>C30-$C$24</f>
+        <v>3.9639999999999675E-3</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
@@ -1084,8 +1084,12 @@
         <v>0.88875599999999999</v>
       </c>
       <c r="D31">
-        <f t="shared" si="16"/>
-        <v>3.8688000000000056E-2</v>
+        <f>B31-$B$24</f>
+        <v>4.2070000000000718E-3</v>
+      </c>
+      <c r="E31">
+        <f>C31-$C$24</f>
+        <v>6.1529999999999641E-3</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
@@ -1098,8 +1102,16 @@
       <c r="C32">
         <v>0.87873100000000004</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D32">
+        <f>B32-$B$24</f>
+        <v>-6.472999999999951E-3</v>
+      </c>
+      <c r="E32">
+        <f>C32-$C$24</f>
+        <v>-3.8719999999999866E-3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>28</v>
       </c>
@@ -1109,8 +1121,16 @@
       <c r="C33">
         <v>0.86588200000000004</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D33">
+        <f>B33-$B$24</f>
+        <v>-5.5830000000000046E-3</v>
+      </c>
+      <c r="E33">
+        <f>C33-$C$24</f>
+        <v>-1.6720999999999986E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>29</v>
       </c>
@@ -1120,8 +1140,16 @@
       <c r="C34">
         <v>0.88029500000000005</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D34">
+        <f>B34-$B$24</f>
+        <v>-3.2399999999999096E-4</v>
+      </c>
+      <c r="E34">
+        <f>C34-$C$24</f>
+        <v>-2.3079999999999767E-3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>30</v>
       </c>
@@ -1131,8 +1159,16 @@
       <c r="C35">
         <v>0.87909599999999999</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D35">
+        <f>B35-$B$24</f>
+        <v>-4.0449999999999653E-3</v>
+      </c>
+      <c r="E35">
+        <f>C35-$C$24</f>
+        <v>-3.5070000000000379E-3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>31</v>
       </c>
@@ -1142,8 +1178,16 @@
       <c r="C36">
         <v>0.88713299999999995</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D36">
+        <f>B36-$B$24</f>
+        <v>-2.1039999999999948E-3</v>
+      </c>
+      <c r="E36">
+        <f>C36-$C$24</f>
+        <v>4.529999999999923E-3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>32</v>
       </c>
@@ -1153,8 +1197,16 @@
       <c r="C37">
         <v>0.87777899999999998</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D37">
+        <f>B37-$B$24</f>
+        <v>-3.2359999999999056E-3</v>
+      </c>
+      <c r="E37">
+        <f>C37-$C$24</f>
+        <v>-4.8240000000000505E-3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>34</v>
       </c>
@@ -1164,8 +1216,16 @@
       <c r="C38">
         <v>0.876309</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D38">
+        <f>B38-$B$24</f>
+        <v>-7.0389999999999064E-3</v>
+      </c>
+      <c r="E38">
+        <f>C38-$C$24</f>
+        <v>-6.2940000000000218E-3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>33</v>
       </c>
@@ -1175,8 +1235,16 @@
       <c r="C39">
         <v>0.87090599999999996</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D39">
+        <f>B39-$B$24</f>
+        <v>-5.9869999999999646E-3</v>
+      </c>
+      <c r="E39">
+        <f>C39-$C$24</f>
+        <v>-1.1697000000000068E-2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>35</v>
       </c>
@@ -1186,8 +1254,16 @@
       <c r="C40">
         <v>0.89281999999999995</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D40">
+        <f>B40-$B$24</f>
+        <v>7.4430000000000884E-3</v>
+      </c>
+      <c r="E40">
+        <f>C40-$C$24</f>
+        <v>1.0216999999999921E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>36</v>
       </c>
@@ -1197,8 +1273,16 @@
       <c r="C41">
         <v>0.88603500000000002</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D41">
+        <f>B41-$B$24</f>
+        <v>5.6630000000000846E-3</v>
+      </c>
+      <c r="E41">
+        <f>C41-$C$24</f>
+        <v>3.4319999999999906E-3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>37</v>
       </c>
@@ -1208,8 +1292,16 @@
       <c r="C42">
         <v>0.89135799999999998</v>
       </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D42">
+        <f>B42-$B$24</f>
+        <v>5.0970000000000182E-3</v>
+      </c>
+      <c r="E42">
+        <f>C42-$C$24</f>
+        <v>8.7549999999999573E-3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>38</v>
       </c>
@@ -1219,8 +1311,16 @@
       <c r="C43">
         <v>0.89242100000000002</v>
       </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D43">
+        <f>B43-$B$24</f>
+        <v>5.0160000000000204E-3</v>
+      </c>
+      <c r="E43">
+        <f>C43-$C$24</f>
+        <v>9.8179999999999934E-3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>39</v>
       </c>
@@ -1230,8 +1330,16 @@
       <c r="C44">
         <v>0.87372300000000003</v>
       </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D44">
+        <f>B44-$B$24</f>
+        <v>-5.6599999999995543E-4</v>
+      </c>
+      <c r="E44">
+        <f>C44-$C$24</f>
+        <v>-8.879999999999999E-3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>40</v>
       </c>
@@ -1241,8 +1349,16 @@
       <c r="C45">
         <v>0.87926099999999996</v>
       </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D45">
+        <f>B45-$B$24</f>
+        <v>-4.8549999999999427E-3</v>
+      </c>
+      <c r="E45">
+        <f>C45-$C$24</f>
+        <v>-3.3420000000000671E-3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>41</v>
       </c>
@@ -1251,6 +1367,14 @@
       </c>
       <c r="C46">
         <v>0.90144199999999997</v>
+      </c>
+      <c r="D46">
+        <f>B46-$B$24</f>
+        <v>1.2864000000000098E-2</v>
+      </c>
+      <c r="E46">
+        <f>C46-$C$24</f>
+        <v>1.8838999999999939E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>